<commit_message>
Oct 27 contract history: add the Arm A floor refusals (IRFC, PNB) [skip render]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/results/S1_fade_oct27_contract_history.xlsx
+++ b/data/results/S1_fade_oct27_contract_history.xlsx
@@ -24,6 +24,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAJFINANCE 920PE" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HINDZINC 540PE" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UNIONBANK 180PE" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRFC 80CE" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PNB 122CE" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:S21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -490,7 +492,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Results day (day 0)</t>
+          <t>Trade day (day 0 / entry day)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -592,7 +594,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -669,7 +671,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>refused: premium below Rs 2 (strike nearest the stock)</t>
+          <t>Arm F fade, refused: premium below Rs 2 (strike nearest the stock)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -727,7 +729,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -804,7 +806,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -881,7 +883,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -958,7 +960,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1035,7 +1037,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1112,7 +1114,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1189,7 +1191,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1266,7 +1268,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1343,7 +1345,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1420,7 +1422,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>refused: premium below Rs 2 (the contract in your screenshot)</t>
+          <t>Arm F fade, refused: premium below Rs 2 (the contract in your screenshot)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1478,7 +1480,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>refused: premium below Rs 2 (strike nearest the stock)</t>
+          <t>Arm F fade, refused: premium below Rs 2 (strike nearest the stock)</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1536,7 +1538,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1607,7 +1609,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>bought</t>
+          <t>Arm F fade, bought</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1678,7 +1680,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>refused: 1 lot too big for the Rs 2 floor (the walk's strike)</t>
+          <t>Arm F fade, refused: 1 lot too big for the Rs 2 floor (the walk's strike)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1712,8 +1714,118 @@
         <v>-44.3</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IRFC 27 Oct 80 Call</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Arm A, refused: premium below Rs 2 (signal 16 Oct, entry day 19 Oct; stock 80.26)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O18" t="n">
+        <v>5</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>-91.09999999999999</v>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PNB 27 Oct 122 Call</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Arm A, refused: 1 lot too big for the Rs 2 floor (signal 19 Oct, entry day 21 Oct; stock 121.89)</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N19" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="O19" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>-23.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Oct 27 contracts first listed on 29 Jul 2026; a strike's first trade day can be later. 20 Oct was a holiday; 21 Oct's NSE file is not out yet. Source: NSE F&amp;O daily bhavcopy.</t>
         </is>
@@ -1753,7 +1865,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 62.15 at 09:15:44, sold 40.55 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 62.15 at 09:15:44, sold 40.55 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2285,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 12.2 at 09:15:44, sold 2.8 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 12.2 at 09:15:44, sold 2.8 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2761,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-19 · bought · bought 2.6 at 09:16:58, sold 0.25 (fade_eod)</t>
+          <t>Trade day: 2026-10-19 · Arm F fade, bought · bought 2.6 at 09:16:58, sold 0.25 (fade_eod)</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3405,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-19 · refused: premium below Rs 2 (the contract in your screenshot)</t>
+          <t>Trade day: 2026-10-19 · Arm F fade, refused: premium below Rs 2 (the contract in your screenshot)</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3741,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-19 · refused: premium below Rs 2 (strike nearest the stock)</t>
+          <t>Trade day: 2026-10-19 · Arm F fade, refused: premium below Rs 2 (strike nearest the stock)</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4133,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-21 · bought · bought 8.15 at 09:15:47, sold 4.9 (fade_stop)</t>
+          <t>Trade day: 2026-10-21 · Arm F fade, bought · bought 8.15 at 09:15:47, sold 4.9 (fade_stop)</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4917,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-21 · bought · bought 5.25 at 09:15:47, sold 4.2 (fade_stop)</t>
+          <t>Trade day: 2026-10-21 · Arm F fade, bought · bought 5.25 at 09:15:47, sold 4.2 (fade_stop)</t>
         </is>
       </c>
     </row>
@@ -5953,7 +6065,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-21 · refused: 1 lot too big for the Rs 2 floor (the walk's strike)</t>
+          <t>Trade day: 2026-10-21 · Arm F fade, refused: 1 lot too big for the Rs 2 floor (the walk's strike)</t>
         </is>
       </c>
     </row>
@@ -6897,6 +7009,1714 @@
       </c>
       <c r="H37" t="n">
         <v>-74.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>IRFC 27 Oct 80 Call</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Trade day: 2026-10-19 · Arm A, refused: premium below Rs 2 (signal 16 Oct, entry day 19 Oct; stock 80.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NSE daily prices, every day it traded from its first trade (2026-09-02) to 2026-10-19. Yellow = day 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Open ₹</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>High ₹</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Low ₹</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Close ₹</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Contracts traded</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Close vs first close %</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Close vs previous %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-1.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.79</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-18.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-15.3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-4.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-23.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>44</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>187</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-48.9</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-32.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>171</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-48.9</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F15" t="n">
+        <v>457</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-46.9</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="F16" t="n">
+        <v>366</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-31.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F17" t="n">
+        <v>205</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-42.4</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-15.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="F18" t="n">
+        <v>297</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-45.6</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-5.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F19" t="n">
+        <v>243</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-38.4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F20" t="n">
+        <v>536</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-53.6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-24.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="F21" t="n">
+        <v>622</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-59.1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1095</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-73.3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-34.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1658</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-69.59999999999999</v>
+      </c>
+      <c r="H23" t="n">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7290</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-64.2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2124</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-74.90000000000001</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-29.8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1081</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-78.2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-13.3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1122</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-73.3</v>
+      </c>
+      <c r="H27" t="n">
+        <v>22.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1007</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-80.90000000000001</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-28.3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1469</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-88.90000000000001</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-41.9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F30" t="n">
+        <v>812</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-88.7</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-76.7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>105.9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2224</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-63.1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2324</v>
+      </c>
+      <c r="G33" t="n">
+        <v>-64</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-2.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3184</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-73.8</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-27.2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="F35" t="n">
+        <v>7503</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-73.09999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>2839</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>-91.09999999999999</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>-66.90000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>PNB 27 Oct 122 Call</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Trade day: 2026-10-21 · Arm A, refused: 1 lot too big for the Rs 2 floor (signal 19 Oct, entry day 21 Oct; stock 121.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NSE daily prices, every day it traded from its first trade (2026-09-01) to 2026-10-19. Yellow = day 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Open ₹</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>High ₹</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Low ₹</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Close ₹</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Contracts traded</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Close vs first close %</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Close vs previous %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-4.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F10" t="n">
+        <v>21</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>40</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-12</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-13.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F12" t="n">
+        <v>31</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F13" t="n">
+        <v>28</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-15.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="F14" t="n">
+        <v>41</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-29.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-18.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F15" t="n">
+        <v>101</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-61.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-45.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F16" t="n">
+        <v>79</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-66.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-13.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F17" t="n">
+        <v>74</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-64</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F18" t="n">
+        <v>87</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-76.40000000000001</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-34.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F19" t="n">
+        <v>98</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-74</v>
+      </c>
+      <c r="H19" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F20" t="n">
+        <v>130</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-78.8</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-18.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F21" t="n">
+        <v>500</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-62.4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>77.40000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F22" t="n">
+        <v>407</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-54.4</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="F23" t="n">
+        <v>303</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-52.4</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F24" t="n">
+        <v>107</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-61.2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-18.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="F25" t="n">
+        <v>266</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-49.6</v>
+      </c>
+      <c r="H25" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F26" t="n">
+        <v>777</v>
+      </c>
+      <c r="G26" t="n">
+        <v>-30.4</v>
+      </c>
+      <c r="H26" t="n">
+        <v>38.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F27" t="n">
+        <v>779</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-64.40000000000001</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-48.9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="F28" t="n">
+        <v>629</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-67.2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-7.9</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5214</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>134.1</v>
       </c>
     </row>
   </sheetData>
@@ -6933,7 +8753,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-15 · bought · bought 2.25 at 15:17:13, sold 2.2 (fade_eod)</t>
+          <t>Trade day: 2026-10-15 · Arm F fade, bought · bought 2.25 at 15:17:13, sold 2.2 (fade_eod)</t>
         </is>
       </c>
     </row>
@@ -7717,7 +9537,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-15 · refused: premium below Rs 2 (strike nearest the stock)</t>
+          <t>Trade day: 2026-10-15 · Arm F fade, refused: premium below Rs 2 (strike nearest the stock)</t>
         </is>
       </c>
     </row>
@@ -9145,7 +10965,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 2.6 at 09:15:44, sold 6.0 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 2.6 at 09:15:44, sold 6.0 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -10237,7 +12057,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 5.95 at 09:15:44, sold 0.9 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 5.95 at 09:15:44, sold 0.9 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -10825,7 +12645,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 3.03 at 09:15:44, sold 2.72 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 3.03 at 09:15:44, sold 2.72 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -11693,7 +13513,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 3.55 at 09:15:44, sold 1.95 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 3.55 at 09:15:44, sold 1.95 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -12169,7 +13989,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 14.5 at 09:15:44, sold 11.8 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 14.5 at 09:15:44, sold 11.8 (fade_late)</t>
         </is>
       </c>
     </row>
@@ -12729,7 +14549,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Results day (day 0): 2026-10-16 · bought · bought 49.45 at 09:15:44, sold 55.75 (fade_late)</t>
+          <t>Trade day: 2026-10-16 · Arm F fade, bought · bought 49.45 at 09:15:44, sold 55.75 (fade_late)</t>
         </is>
       </c>
     </row>

</xml_diff>